<commit_message>
Final ranking: Landmark reconciliation to #2 per Codex review
Accepted one Codex recommendation: moved Landmark QB reconciliation
from #4 to #2 (overdue, blocks March close chain). All other rankings
kept per Roper's judgment. Codex review request and response preserved.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Signature Integration Milestone View — Roper Update 2026-04-05.xlsx
+++ b/Signature Integration Milestone View — Roper Update 2026-04-05.xlsx
@@ -16,9 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yy"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="25">
     <font>
@@ -1319,7 +1318,7 @@
         </is>
       </c>
       <c r="I18" s="31" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19">
@@ -1391,7 +1390,7 @@
         </is>
       </c>
       <c r="I20" s="31" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="21">
@@ -1720,7 +1719,7 @@
         </is>
       </c>
       <c r="I33" s="31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="34">
@@ -2123,7 +2122,7 @@
         </is>
       </c>
       <c r="I48" s="31" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="49">
@@ -2226,7 +2225,7 @@
         </is>
       </c>
       <c r="I51" s="31" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52">
@@ -2356,7 +2355,7 @@
         </is>
       </c>
       <c r="I55" s="31" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="56">
@@ -2671,7 +2670,7 @@
         </is>
       </c>
       <c r="I66" s="31" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="67">
@@ -2793,7 +2792,7 @@
         </is>
       </c>
       <c r="I70" s="31" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="71">
@@ -2815,6 +2814,8 @@
         <v>46161.70833332176</v>
       </c>
     </row>
+    <row r="72"/>
+    <row r="73"/>
     <row r="74">
       <c r="A74" s="33" t="inlineStr">
         <is>
@@ -2897,7 +2898,7 @@
         </is>
       </c>
       <c r="I76" s="34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="77">
@@ -2975,7 +2976,7 @@
         </is>
       </c>
       <c r="I78" s="34" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="79">
@@ -3014,7 +3015,7 @@
         </is>
       </c>
       <c r="I79" s="34" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="80">
@@ -3053,7 +3054,7 @@
         </is>
       </c>
       <c r="I80" s="34" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="81">
@@ -3092,7 +3093,7 @@
         </is>
       </c>
       <c r="I81" s="34" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="82">
@@ -3131,7 +3132,7 @@
         </is>
       </c>
       <c r="I82" s="34" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="83">
@@ -3170,7 +3171,7 @@
         </is>
       </c>
       <c r="I83" s="34" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="84">
@@ -3209,7 +3210,7 @@
         </is>
       </c>
       <c r="I84" s="34" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="85">
@@ -3251,6 +3252,8 @@
         <v>19</v>
       </c>
     </row>
+    <row r="86"/>
+    <row r="87"/>
     <row r="88">
       <c r="A88" s="33" t="inlineStr">
         <is>
@@ -3549,6 +3552,8 @@
       </c>
       <c r="I97" s="34" t="n"/>
     </row>
+    <row r="98"/>
+    <row r="99"/>
     <row r="100">
       <c r="A100" s="33" t="inlineStr">
         <is>

</xml_diff>